<commit_message>
Correct the dictionary: deal-type ownership, active workflow counts, renewals, Apex
Also adds the statements-to-confirm list, backlog item 21 and softens the
Ironclad re-sync note in the object scope.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018HFwLkiuTro1Y9Y8fCndHQ
</commit_message>
<xml_diff>
--- a/docs/data-library/Passport_Process_and_Data_Dictionary_2026-10-19.xlsx
+++ b/docs/data-library/Passport_Process_and_Data_Dictionary_2026-10-19.xlsx
@@ -33,7 +33,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Process Cards'!$A$4:$H$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Field Mapping Starter'!$A$5:$H$35</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Cleanup Backlog'!$A$5:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Cleanup Backlog'!$A$5:$G$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -926,7 +926,7 @@
     <row r="5" ht="75" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Ownership and cadence. Client Success Rep and Secondary Client Success Rep are lookups on the Account (the CS Assignment flow and a validation rule keep rep changes to managers). Client Tier is a formula on Recurring NS revenue: Tier 1 above $800k, Tier 2 $300k to $800k, Tier 3 $100k to $300k, Tier 4 $30k to $100k, Tier 5 below. Required Check-in Frequency follows the tier (Bi-weekly, Monthly, Bi-Monthly, Bi-Annual), Last Call Date is stamped from logged calls and meetings, and Check-in Status reads On Track, Due Soon or Overdue; a weekly email lists overdue accounts. CS Segmentation (Retention, Growth, Growth - Enforcement, Growth - Payments, Channel) is set automatically from which product families the account holds, with a manual override.</t>
+          <t>Ownership and cadence. Client Success Rep and Secondary Client Success Rep are lookups on the Account; a validation rule restricts rep changes to managers. Client Tier is a formula on Recurring NS revenue: Tier 1 above $800k, Tier 2 $300k to $800k, Tier 3 $100k to $300k, Tier 4 $30k to $100k, Tier 5 below. Required Check-in Frequency follows the tier (Bi-weekly, Monthly, Bi-Monthly, Bi-Annual), Last Call Date is stamped from logged calls and meetings, and Check-in Status reads On Track, Due Soon or Overdue; a weekly email lists overdue accounts. CS Segmentation (Retention, Growth, Growth - Enforcement, Growth - Payments, Channel) is set automatically from which product families the account holds, with a manual override.</t>
         </is>
       </c>
     </row>
@@ -947,14 +947,14 @@
     <row r="8" ht="60" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Churn. Churn is recorded on the Account: Status changes to Former, Churn Date and Churn Reason are set (Lost RFP, Product Functionality, Support/Service Dissatisfaction, Price, City Transition to Channel, Channel Transition to City, Account Clean Up, Other), a Churn Explanation is required on the change, and a workflow rule snapshots Recurring NS revenue into Churn Recurring Revenue at that moment, which is the lost-revenue figure. An email announces the churn. Former customers: 478, of which 85 churned in 2023 to 2026 with a date; the remaining 394 are legacy records with no churn date or reason, mostly from a 2026 cleanup.</t>
+          <t>Churn. Churn is recorded on the Account: Status changes to Former, Churn Date and Churn Reason are set (Lost RFP, Product Functionality, Support/Service Dissatisfaction, Price, City Transition to Channel, Channel Transition to City, Account Clean Up, Other), a Churn Explanation is required on the change, and a workflow rule snapshots Recurring NS revenue into Churn Recurring Revenue at that moment, which is the lost-revenue figure. An email announces the churn. Former customers: 478, of which 85 churned in 2023 to 2026 with a date; the remaining 394 are legacy records with no churn date or reason.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Implementation. Between close and launch, Opportunity Products carry Implementation Status, Implementation Engineer, Project Manager and launch dates; Implementation Status Tracker records (5,222) and Implementation At-Risk Journeys (164) track delivery risk with their own workflow email alerts. Cases on record types Request Solutions Engineering (373 in the last 12 months) and SFDC Change Request (329) carry internal requests to Solutions Engineering and RevOps; customer support itself runs outside Salesforce (Intercom and Helpshift), with every new Account pushed to Intercom automatically.</t>
+          <t>Implementation. Between close and launch, Opportunity Products carry Implementation Status, Implementation Engineer, Project Manager and launch dates; Implementation Status Tracker records (5,222) and Implementation At-Risk Journeys (164) track delivery risk with their own workflow email alerts. Cases on record types Request Solutions Engineering (373 in the last 12 months) and SFDC Change Request (329) carry internal requests to Solutions Engineering and RevOps; customer support itself runs outside Salesforce (Intercom), with every new Account pushed to Intercom automatically.</t>
         </is>
       </c>
     </row>
@@ -1634,10 +1634,10 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>The org runs on declarative automation: 66 active record-triggered flows, 6 scheduled flows, 3 screen flows, 58 classic workflow rules still active, 9 Apex triggers (5 of them from the roll-up packages) and no custom Apex of Passport's own beyond those triggers. Half of the flows sit on the Opportunity. Fourteen active flows send to a named mailbox or person or carry a hard-coded user or queue ID; those are the ones a merge or a departure breaks first.</t>
+          <t>The org runs on declarative automation: 66 active record-triggered flows, 6 scheduled flows, 3 screen flows, 58 classic workflow rules still active, 9 Apex triggers (5 of them generated by the roll-up tool) and 54 Apex classes of Passport's own, all legacy (old customer-portal and public knowledge-base controllers and trigger tests); none of the seven processes depends on custom code. Half of the flows sit on the Opportunity. Fourteen active flows send to a named mailbox or person or carry a hard-coded user or queue ID; those are the ones a merge or a departure breaks first.</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Workflow rules</t>
+          <t>Active workflow rules</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1663,7 +1663,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="52" customHeight="1">
+    <row r="7" ht="78" customHeight="1">
       <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Opportunity</t>
@@ -1676,16 +1676,16 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Stage and close notifications (Slack and email), renewal creation, MEDDIC mirror, stamps and counters, Capture Strategy auto-close</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="39" customHeight="1">
+          <t>Stage and close notifications (Slack and email), renewal creation, MEDDIC mirror, stamps and counters, Capture Strategy auto-close; the two workflow rules are a renewal reminder and a CS-rep assignment email</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
       <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Case</t>
@@ -1698,188 +1698,188 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>33</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>FOIA process (7 flows), SE request routing, status trackers and change-request feed posts</t>
+          <t>FOIA process (7 flows) and SE request routing; the workflow rules are status-change emails, queue routing and date stamps for the internal request desks</t>
         </is>
       </c>
     </row>
     <row r="9" ht="39" customHeight="1">
       <c r="B9" s="7" t="inlineStr">
         <is>
+          <t>Email Message</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Case response handling: first-contact stamp, reopen on customer reply, auto-response flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="65" customHeight="1">
+      <c r="B10" s="7" t="inlineStr">
+        <is>
           <t>Account</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>Intercom push, CS assignment, segmentation, target revenue, churn date and churn revenue capture, at-risk alerts</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="39" customHeight="1">
-      <c r="B10" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>Intercom push, CS assignment, segmentation, target revenue, churn date; the workflow rules capture churn revenue, email the churn, stamp At-Risk Date and set Status to Current on the first win</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="39" customHeight="1">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>At-Risk Journey</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>One-open-journey guard, account mirror sync, open / de-risk / predicted-churn emails</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="B11" s="7" t="inlineStr">
+    <row r="12" ht="52" customHeight="1">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Opportunity Product</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>Launch date to Asset, product cost, implementation-cancelled email</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="B12" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Launch date to Asset, product cost, implementation-cancelled email; the workflow rules track launch-date changes and send the launched notice</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="26" customHeight="1">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Asset</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Launch date from the deal line, Multi-App</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="39" customHeight="1">
-      <c r="B13" s="7" t="inlineStr">
+    <row r="14" ht="39" customHeight="1">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Capture Strategy</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
-          <t>Slack on create; date stamps and stage moves on submission, shortlist and pricing review</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Lead</t>
-        </is>
-      </c>
-      <c r="C14" s="7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>Best Matched Account; territory by state; inbound date</t>
+          <t>Slack on create; date stamps on submission, shortlist and pricing review; stage to Ready for Submission</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="B15" s="7" t="inlineStr">
         <is>
+          <t>Lead</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Best Matched Account; territory by state (7 rules); inbound date stamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="26" customHeight="1">
+      <c r="B16" s="7" t="inlineStr">
+        <is>
           <t>MEDDIC, Deal Desk Approval, Event, Task</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>1 each</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Opportunity created date stamp, approval email, Last Call Date on the Account</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Implementation At-Risk Journey</t>
-        </is>
-      </c>
-      <c r="C16" s="7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Implementation risk email alerts</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J35"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2771,10 +2771,10 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
+    <row r="5" ht="30" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Data quality Passport is already working on.</t>
+          <t>Statements to confirm before relying on them. Most of this document is read from the org. The following are Revenue Operations' interpretation and should be confirmed with the named owners before they are treated as fact:</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Procurement Method blank on 752 of 805 recent wins; a correction list is in progress with Proposal Operations.</t>
+          <t>The plain-language definitions of the deal Types (Revenue Operations). Ownership by Type is measured; the wording is not.</t>
         </is>
       </c>
     </row>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>394 former customers without churn date or reason; 213 without a date at all.</t>
+          <t>How pricing exceptions are approved now that the Deal Desk approval process is obsolete (Revenue Operations).</t>
         </is>
       </c>
     </row>
@@ -2810,7 +2810,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>312 open deals in retired stages; 270 picklist values present in data but no longer defined; 515 custom fields filled on less than 1 percent of records.</t>
+          <t>What the Celigo connector sends to NetSuite on a closed-won deal, beyond the monthly revenue it writes back (Finance systems).</t>
         </is>
       </c>
     </row>
@@ -2822,7 +2822,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>379 inactive users still own 60 percent of opportunities; ownership was never reassigned at offboarding.</t>
+          <t>The source of the 93,600 automatically logged email tasks, assumed to be the Gmail integration's automatic logging (Revenue Operations).</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Asset contract end dates not advanced after auto-renewal (worked around by the Renewal Date formula); renewal term unknown.</t>
+          <t>Whether Ironclad can re-push workflow and contract records into another org (Ironclad administrator).</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Ironclad Contract repository unsynced since 2021; keyed backfill planned.</t>
+          <t>The purpose of the Fivetran, Zapier and Pursuit connections, inferred from their names and login patterns.</t>
         </is>
       </c>
     </row>
@@ -2858,11 +2858,11 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>13 validation rules and 2 flows carry hard-coded user or profile IDs; several notification flows name individuals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1">
+          <t>Everything said about Arrive's model comes from meeting notes, not from their org.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Storage: 1.49 million pipeline snapshot rows and 1.29 million tasks dominate data storage; 13.6 GB of legacy Attachments.</t>
+          <t>Field dispositions in the workbook checked presence on 24 core page layouts only; the other layouts, list views, reports and email templates were not checked, so a Retire candidate must be confirmed by its owner before removal.</t>
         </is>
       </c>
     </row>
@@ -2882,18 +2882,18 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>SOAP API login is used by one integration (Celigo) and must move to OAuth before Summer '27.</t>
+          <t>The three-year cut-offs in the object scope and the grouping rule behind the duplicate scan are proposals, not policy.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Structural points for a combined org.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+          <t>Data quality Passport is already working on.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2901,11 +2901,11 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>One account per agency. Passport keys everything to a single Account per customer, with one team selling four product lines. Arrive separates on-street and off-street business units with separate deals and reps per city. A combined model has to decide whether that split lives on the Account (two accounts per city), on the Opportunity (a business-unit field), or on the product line. Passport's product family already carries most of the on-street versus off-street meaning (Parking and Enforcement are on-street; gated garages would be a new family).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>Procurement Method blank on 752 of 805 recent wins; a correction list is in progress with Proposal Operations.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2913,11 +2913,11 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Deal Type semantics. New Customer, Cross-Sell, Upsell, Revenue Enhancement and Renewal drive the rules, the notifications and the renewal flow. Mapping Arrive's deal types onto these (or the reverse) decides which automation survives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>394 former customers without churn date or reason; 213 without a date at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2925,11 +2925,11 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Stage path and gates. Nine stages with field gates for new business; a four-stage renewal path. The gates encode Passport's sales method (MEDDIC at Discovery, SE review, scoped proposal, award evidence) and are the main source of data completeness.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>312 open deals in retired stages; 270 picklist values present in data but no longer defined; 515 custom fields filled on less than 1 percent of records.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2937,11 +2937,11 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Bid tracking. Capture Strategy holds the bid lifecycle with validation; Arrive's bid management is a North American spreadsheet. The spreadsheet's statuses, stage definitions, leads, products, agencies and due dates map onto Capture Strategy fields almost one to one; the comparison needs the spreadsheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="30" customHeight="1">
+          <t>379 inactive users still own 60 percent of opportunities; ownership was never reassigned at offboarding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2949,11 +2949,11 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Contract to asset. Passport links contract (Ironclad) to deal to installed product with dates and a rolling renewal date. The Asset is the installed-base record and feeds segmentation and product flags.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="30" customHeight="1">
+          <t>Asset contract end dates not advanced after auto-renewal (worked around by the Renewal Date formula); renewal term unknown.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2961,7 +2961,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Revenue feed. Monthly NetSuite revenue by customer and product family on the Account. A combined org needs one ERP feed with the same grain or a clear statement of two.</t>
+          <t>Ironclad Contract repository unsynced since 2021; keyed backfill planned.</t>
         </is>
       </c>
     </row>
@@ -2973,11 +2973,11 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Marketing. Both companies run HubSpot; Arrive's contract is separate from go-to-market for a year, so two HubSpot portals may feed one Salesforce for a period.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="30" customHeight="1">
+          <t>13 validation rules and 2 flows carry hard-coded user or profile IDs; several notification flows name individuals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2985,11 +2985,11 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Client Success. MEDDIC on the account, check-in cadence by tier, formal at-risk journeys and churn capture are mature and should be preserved in whichever org survives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="30" customHeight="1">
+          <t>Storage: 1.49 million pipeline snapshot rows and 1.29 million tasks dominate data storage; 13.6 GB of legacy Attachments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>•</t>
@@ -2997,110 +2997,230 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Package debt. 23 managed packages own 70 percent of the fields; several (Helpshift, Freshdesk, Responsive, SalesforceIQ, Periscope) are retired and can be uninstalled before any migration.</t>
+          <t>SOAP API login is used by one integration (Celigo) and must move to OAuth before Summer '27.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1">
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>Structural points for a combined org.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>One account per agency. Passport keys everything to a single Account per customer, with one team selling four product lines. Arrive separates on-street and off-street business units with separate deals and reps per city. A combined model has to decide whether that split lives on the Account (two accounts per city), on the Opportunity (a business-unit field), or on the product line. Passport's product family already carries most of the on-street versus off-street meaning (Parking and Enforcement are on-street; gated garages would be a new family).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Deal Type semantics. New Customer, Cross-Sell, Upsell, Revenue Enhancement and Renewal drive the rules, the notifications and the renewal flow. Mapping Arrive's deal types onto these (or the reverse) decides which automation survives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="30" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Stage path and gates. Nine stages with field gates for new business; a four-stage renewal path. The gates encode Passport's sales method (MEDDIC at Discovery, SE review, scoped proposal, award evidence) and are the main source of data completeness.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Bid tracking. Capture Strategy holds the bid lifecycle with validation; Arrive's bid management is a North American spreadsheet. The spreadsheet's statuses, stage definitions, leads, products, agencies and due dates map onto Capture Strategy fields almost one to one; the comparison needs the spreadsheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>Contract to asset. Passport links contract (Ironclad) to deal to installed product with dates and a rolling renewal date. The Asset is the installed-base record and feeds segmentation and product flags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Revenue feed. Monthly NetSuite revenue by customer and product family on the Account. A combined org needs one ERP feed with the same grain or a clear statement of two.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Marketing. Both companies run HubSpot; Arrive's contract is separate from go-to-market for a year, so two HubSpot portals may feed one Salesforce for a period.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Client Success. MEDDIC on the account, check-in cadence by tier, formal at-risk journeys and churn capture are mature and should be preserved in whichever org survives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Package debt. 23 managed packages own 70 percent of the fields; several (Helpshift, Freshdesk, Responsive, SalesforceIQ, Periscope) are retired and can be uninstalled before any migration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
           <t>Questions for Arrive's team.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr">
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="5" t="inlineStr"/>
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>1. How is an agency that buys both on-street and off-street services represented: one account or two, and how do deals, contracts and installed products attach?</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customHeight="1">
-      <c r="A27" s="5" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr">
+    <row r="37" ht="15" customHeight="1">
+      <c r="A37" s="5" t="inlineStr"/>
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>2. What are the deal types and stage definitions in the consolidated Arrive org, and which fields are required at each stage?</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1">
-      <c r="A28" s="5" t="inlineStr"/>
-      <c r="B28" s="4" t="inlineStr">
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="5" t="inlineStr"/>
+      <c r="B38" s="4" t="inlineStr">
         <is>
           <t>3. Where does the bid tracker live now, what are its statuses and stage definitions, and who owns a bid from intake to award?</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1">
-      <c r="A29" s="5" t="inlineStr"/>
-      <c r="B29" s="4" t="inlineStr">
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="5" t="inlineStr"/>
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>4. How are signed contracts linked to deals and to installed products or subscriptions, and where do contract dates and renewal terms live?</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="5" t="inlineStr"/>
-      <c r="B30" s="4" t="inlineStr">
+    <row r="40" ht="15" customHeight="1">
+      <c r="A40" s="5" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>5. What is the revenue source of record, at what grain (customer, product, site) and how often does it refresh into Salesforce?</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="15" customHeight="1">
-      <c r="A31" s="5" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr">
+    <row r="41" ht="15" customHeight="1">
+      <c r="A41" s="5" t="inlineStr"/>
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>6. How is renewal handled: automatic renewal deals, a contract object, or subscription records?</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1">
-      <c r="A32" s="5" t="inlineStr"/>
-      <c r="B32" s="4" t="inlineStr">
+    <row r="42" ht="15" customHeight="1">
+      <c r="A42" s="5" t="inlineStr"/>
+      <c r="B42" s="4" t="inlineStr">
         <is>
           <t>7. What does client success record: health, risk, churn reasons, QBR cadence?</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1">
-      <c r="A33" s="5" t="inlineStr"/>
-      <c r="B33" s="4" t="inlineStr">
+    <row r="43" ht="15" customHeight="1">
+      <c r="A43" s="5" t="inlineStr"/>
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>8. Which identifiers travel across systems (customer IDs, product codes, agency codes) that a merged account and product catalogue would need to keep?</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="5" t="inlineStr"/>
-      <c r="B34" s="4" t="inlineStr">
+    <row r="44" ht="15" customHeight="1">
+      <c r="A44" s="5" t="inlineStr"/>
+      <c r="B44" s="4" t="inlineStr">
         <is>
           <t>9. How does the HubSpot integration work today (which objects sync, which portal is primary) and what happens at the end of the one-year contract?</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="30" customHeight="1">
-      <c r="A35" s="5" t="inlineStr"/>
-      <c r="B35" s="4" t="inlineStr">
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="5" t="inlineStr"/>
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>10. Which org is expected to survive in 2027, and what is the appetite for rebuilding clunky objects (Passport's Capture Strategy among them) rather than migrating them as they are?</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="43">
     <mergeCell ref="B11:J11"/>
+    <mergeCell ref="B42:J42"/>
     <mergeCell ref="B14:J14"/>
     <mergeCell ref="B17:J17"/>
     <mergeCell ref="B23:J23"/>
     <mergeCell ref="B8:J8"/>
     <mergeCell ref="B13:J13"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B44:J44"/>
     <mergeCell ref="B29:J29"/>
     <mergeCell ref="B19:J19"/>
     <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B37:J37"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B28:J28"/>
+    <mergeCell ref="B40:J40"/>
     <mergeCell ref="B9:J9"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="B24:J24"/>
@@ -3109,8 +3229,11 @@
     <mergeCell ref="B33:J33"/>
     <mergeCell ref="B5:J5"/>
     <mergeCell ref="B20:J20"/>
+    <mergeCell ref="B45:J45"/>
+    <mergeCell ref="B36:J36"/>
     <mergeCell ref="B32:J32"/>
     <mergeCell ref="B26:J26"/>
+    <mergeCell ref="B41:J41"/>
     <mergeCell ref="B35:J35"/>
     <mergeCell ref="B4:J4"/>
     <mergeCell ref="B16:J16"/>
@@ -3120,7 +3243,9 @@
     <mergeCell ref="B31:J31"/>
     <mergeCell ref="B18:J18"/>
     <mergeCell ref="B27:J27"/>
+    <mergeCell ref="B43:J43"/>
     <mergeCell ref="B12:J12"/>
+    <mergeCell ref="B39:J39"/>
     <mergeCell ref="B21:J21"/>
     <mergeCell ref="B2:J2"/>
   </mergeCells>
@@ -3575,7 +3700,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>AE (Standard), CSM (Renewal)</t>
+          <t>AE for New Customer and Cross-Sell; CSM for Upsell, Revenue Enhancement and Renewal</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -4969,7 +5094,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5779,14 +5904,51 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Revenue Enhancement Type blank on 164 of 175 recent Revenue Enhancement deals; the picklist already carries fee-increase values the price-increase work can reuse</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Client Success + RevOps</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A5:G25"/>
+  <autoFilter ref="A5:G26"/>
   <mergeCells count="2">
     <mergeCell ref="A3:G3"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="G6:G225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G6:G226" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Blocked,Parked,Done"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6062,7 +6224,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="52" customHeight="1">
+    <row r="14" ht="65" customHeight="1">
       <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Activity</t>
@@ -6070,7 +6232,7 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>1.29 million Tasks, 18,667 Events; 178,000 tasks logged in the last 12 months, 94 percent of them by HubSpot and automatic email and calendar capture</t>
+          <t>1.29 million Tasks, 18,667 Events; 178,000 tasks logged in the last 12 months: 72,700 from the HubSpot integration, 93,600 automatically logged emails, about 10,000 typed by people</t>
         </is>
       </c>
     </row>
@@ -6101,7 +6263,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Sales (Account Executives, Channel reps, Solutions Engineers): Opportunities on the Standard record type, Leads once qualified.</t>
+          <t>Sales (Account Executives, Channel reps, Solutions Engineers): New Customer and Cross-Sell opportunities, Leads once qualified.</t>
         </is>
       </c>
     </row>
@@ -6125,7 +6287,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Client Success (CSMs, CSEs, Agents): Accounts after launch, Renewal opportunities, MEDDIC and At-Risk Journeys, Cases.</t>
+          <t>Client Success (CSMs, CSEs, Agents): Accounts after launch; Upsell, Revenue Enhancement and Renewal opportunities; MEDDIC and At-Risk Journeys; Cases.</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6323,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Finance: reads NetSuite revenue on the Account; writes nothing by hand.</t>
+          <t>Finance: consumes the NetSuite revenue written to the Account by the Celigo feed.</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6801,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Region: eight workflow rules set the Sales Territory from the state or province (Canada, East, Midwest, Northeast, Northwest, Southeast, Southwest, West).</t>
+          <t>Region: seven workflow rules set the Sales Territory from the state or province (Canada, East, Midwest, Northeast, Northwest, Southeast, Southwest).</t>
         </is>
       </c>
     </row>
@@ -7005,7 +7167,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>All sales-led deals</t>
+          <t>Sales-led and Client-Success-led deals on one stage path</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -7085,10 +7247,10 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="45" customHeight="1">
+    <row r="12" ht="75" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Type definitions as the business uses them: New Customer is the first product at an account that has never bought; Cross-Sell is a new product line at an existing customer; Upsell is more volume, modules or hardware on a product the customer already has; Revenue Enhancement is a price, fee or term change closed by Client Success; Renewal is the contract renewal created automatically at each close (Process 5).</t>
+          <t>Type definitions as the business uses them (the wording is Revenue Operations' reading and should be confirmed; the ownership figures are measured): New Customer is the first product at an account that has never bought; Cross-Sell is a new product line at an existing customer; Upsell is more volume, modules or hardware on a product the customer already has; Revenue Enhancement is a price, fee or term change closed by Client Success; Renewal is the contract renewal created automatically at each close (Process 5). Sales owns New Customer and Cross-Sell deals; Client Success owns Upsell, Revenue Enhancement and Renewal deals, and closed 76 of the 84 Upsells and 112 of the 115 Revenue Enhancements won in the last 12 months.</t>
         </is>
       </c>
     </row>
@@ -7300,7 +7462,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Approvals: Deal Desk Approval records (29 on file) request leadership sign-off for non-standard pricing; the approval process itself is obsolete and sign-off now happens by email. Travel Approval Requests still use an active approval process.</t>
+          <t>Approvals: Deal Desk Approval records (29 on file) request leadership sign-off for non-standard pricing; the approval process itself is obsolete, and Salesforce does not record how pricing exceptions are approved today. Travel Approval Requests still use an active approval process.</t>
         </is>
       </c>
     </row>
@@ -7406,10 +7568,10 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
+    <row r="8" ht="60" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>2. Close. Closed Won fires the announcements, the Slack post, the renewal creation (Process 5), the Capture Strategy auto-close (Process 2), the account roll-ups (Customer Acquisition Date = earliest won Close Date, Won Opp Count, Amount Sum) and the account Status change to Current. The NetSuite connector (Celigo) reads closed-won deals for billing setup; re-saving a closed deal re-fires it, which is one reason closed deals are locked.</t>
+          <t>2. Close. Closed Won fires the announcements, the Slack post, the renewal creation (Process 5), the Capture Strategy auto-close (Process 2), the account roll-ups (Customer Acquisition Date = earliest won Close Date, Won Opp Count, Amount Sum) and the account Status change to Current. The NetSuite connector (Celigo) is triggered by closed-won deals (what it sends to NetSuite is to be confirmed with Finance systems); re-saving a closed deal re-fires it, which is one reason closed deals are locked.</t>
         </is>
       </c>
     </row>
@@ -7634,7 +7796,7 @@
     <row r="10" ht="45" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Before September 2026 the flow dated every renewal from asset contract dates, which pushed multi-year contracts three or more years out; the open renewals were re-dated by hand when the rule changed. About a third of renewals in the last 12 months were still created by people (Client Success and RevOps) rather than the flow, mostly for accounts whose chain pre-dates it.</t>
+          <t>Before September 2026 the flow dated every renewal from asset contract dates, which pushed multi-year contracts three or more years out; the open renewals were re-dated by hand when the rule changed. The flow always sets Original Opportunity; 292 of the 648 renewals created in the last 12 months have no such link, so a sizeable share are still created by hand.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Combine the dictionary and data library into one 44-tab workbook; blank the Racine amounts
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018HFwLkiuTro1Y9Y8fCndHQ
</commit_message>
<xml_diff>
--- a/docs/data-library/Passport_Process_and_Data_Dictionary_2026-10-19.xlsx
+++ b/docs/data-library/Passport_Process_and_Data_Dictionary_2026-10-19.xlsx
@@ -1186,7 +1186,7 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Lead Source Partner Referral; opened in Discovery at $30k, re-estimated to $130k in July 2025</t>
+          <t>Lead Source Partner Referral; opened in Discovery in June 2025, estimate revised upward in July 2025</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Amount $209,186: $196,931 recurring (Citation Management, Unified Payments) and $12,255 one-time (handhelds, printers, paper, implementation fee); Why Passport written; Procurement Method Direct; 426-day sales cycle</t>
+          <t>Amount about 94 percent recurring (Citation Management, Unified Payments) and 6 percent one-time (handhelds, printers, paper, implementation fee); Why Passport written; Procurement Method Direct; 426-day sales cycle</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">

</xml_diff>